<commit_message>
Remove warning icons from the model text
Client instruction. 49 warning triangles and 1 red circle removed from the
Assumptions and Model note columns. Nothing else changed - the notes already
carry their emphasis in capitals, so no meaning is lost, and the workbook is
now pure ASCII in every cell.

Done as a literal two-character replacement rather than a regex. A first
attempt used a tidy-up regex to collapse the whitespace left behind, and it
matched across newlines, joining code lines and breaking the build. The
narrower edit cannot touch line structure at all.

Verified by scanning every cell of the recalculated workbook for characters
above U+2000: none remain. Y7 revenue unchanged at 3,906,337.

108/108 checks pass, 4,765 formulas, 0 errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model.xlsx
+++ b/deliverables/4-revenue-modeling/tools/Aurumix_Revenue_Model.xlsx
@@ -1381,7 +1381,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RE-PRICED 2026-08-21 from USD 120/yr. THE OLD PRICE WAS ABOVE TRUST &amp; WILL'S PREMIUM US MEMBERSHIP (USD 49/yr) AND WAS 33% OF EVERYTHING THE CUSTOMER SAVES IN A YEAR - a USD 30/month saver puts away USD 360, and we were charging 120 of it. THE INDUSTRY MODEL IS A ONE-OFF FEE PLUS A SMALL ANNUAL UPDATE LAYER, and it is the annual layer this row represents: Trust &amp; Will USD 199 one-off + USD 49/yr; Farewill GBP 100 + GBP 10/yr; Epilogue C$139 with NO subscription at all; other platforms renew updates at ~C$4.50/yr. Formal UAE will registration is a different product entirely and one-off - DIFC AED 10,000 single / 15,000 mirror, Abu Dhabi Civil Court AED 950 as the cheapest formal route. Indian online wills run INR 500-4,000 basic. Family add-ons on finance apps are usually BUNDLED FREE; where charged it is USD 5-15/month for a WHOLE HOUSEHOLD (Monarch 99.99/yr, Zeta 59.99/yr, Greenlight 5.99/mo). SET AT USD 50/yr, client instruction 2026-08-21. That is essentially TRUST &amp; WILL'S USD 49/yr MEMBERSHIP - a defensible anchor in that it matches the best-known product in the category, but ⚠ NOTE WHOSE PRODUCT IT IS: Trust &amp; Will sells to US customers who paid 199-599 up front for an estate plan, not to a migrant worker saving USD 30 a month. At 50 the plan is 14% OF EVERYTHING THE CUSTOMER SAVES IN A YEAR, against 10% at 36 and 33% at the original 120. It is no longer absurd, but it is priced at a developed-market benchmark for an emerging-market customer, and that is the line an adviser would push on. ⚠ A ONE-OFF SETUP FEE IS NOT MODELLED - if the client wants the full industry structure, that is a second row, not a bigger number here. CITED comparators, ASSUMPTION on the point in the range.</t>
+          <t>RE-PRICED 2026-08-21 from USD 120/yr. THE OLD PRICE WAS ABOVE TRUST &amp; WILL'S PREMIUM US MEMBERSHIP (USD 49/yr) AND WAS 33% OF EVERYTHING THE CUSTOMER SAVES IN A YEAR - a USD 30/month saver puts away USD 360, and we were charging 120 of it. THE INDUSTRY MODEL IS A ONE-OFF FEE PLUS A SMALL ANNUAL UPDATE LAYER, and it is the annual layer this row represents: Trust &amp; Will USD 199 one-off + USD 49/yr; Farewill GBP 100 + GBP 10/yr; Epilogue C$139 with NO subscription at all; other platforms renew updates at ~C$4.50/yr. Formal UAE will registration is a different product entirely and one-off - DIFC AED 10,000 single / 15,000 mirror, Abu Dhabi Civil Court AED 950 as the cheapest formal route. Indian online wills run INR 500-4,000 basic. Family add-ons on finance apps are usually BUNDLED FREE; where charged it is USD 5-15/month for a WHOLE HOUSEHOLD (Monarch 99.99/yr, Zeta 59.99/yr, Greenlight 5.99/mo). SET AT USD 50/yr, client instruction 2026-08-21. That is essentially TRUST &amp; WILL'S USD 49/yr MEMBERSHIP - a defensible anchor in that it matches the best-known product in the category, but NOTE WHOSE PRODUCT IT IS: Trust &amp; Will sells to US customers who paid 199-599 up front for an estate plan, not to a migrant worker saving USD 30 a month. At 50 the plan is 14% OF EVERYTHING THE CUSTOMER SAVES IN A YEAR, against 10% at 36 and 33% at the original 120. It is no longer absurd, but it is priced at a developed-market benchmark for an emerging-market customer, and that is the line an adviser would push on. A ONE-OFF SETUP FEE IS NOT MODELLED - if the client wants the full industry structure, that is a second row, not a bigger number here. CITED comparators, ASSUMPTION on the point in the range.</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ADDED 2026-08-21, client instruction. Charged per named beneficiary BEYOND THE FIRST, which the plan includes - the standard shape for this kind of add-on, and the reason the formula carries a MAX(0, n-1) rather than charging every beneficiary. ⚠ NO COMPARABLE EXISTS: will services price PER WILL, not per beneficiary. DIFC charges more for a MIRROR will (two people) and more again for guardianship, but nobody publishes a per-beneficiary tariff. So this is priced on COST RECOVERY, which is the defensible basis available: every named beneficiary needs identity capture and AML screening, and Sumsub screening already sits in this model at ~USD 1.85 per check in the redemption cost memo. USD 6/yr covers that with margin without becoming a second subscription. DELIBERATELY SMALL. At 1.5 chargeable beneficiaries it adds USD 9/yr to a USD 50 plan - an 18% uplift on a stream worth ~3.5% of revenue, so it cannot move the model and should not be tuned to try. ASSUMPTION on a cost-recovery basis.</t>
+          <t>ADDED 2026-08-21, client instruction. Charged per named beneficiary BEYOND THE FIRST, which the plan includes - the standard shape for this kind of add-on, and the reason the formula carries a MAX(0, n-1) rather than charging every beneficiary. NO COMPARABLE EXISTS: will services price PER WILL, not per beneficiary. DIFC charges more for a MIRROR will (two people) and more again for guardianship, but nobody publishes a per-beneficiary tariff. So this is priced on COST RECOVERY, which is the defensible basis available: every named beneficiary needs identity capture and AML screening, and Sumsub screening already sits in this model at ~USD 1.85 per check in the redemption cost memo. USD 6/yr covers that with margin without becoming a second subscription. DELIBERATELY SMALL. At 1.5 chargeable beneficiaries it adds USD 9/yr to a USD 50 plan - an 18% uplift on a stream worth ~3.5% of revenue, so it cannot move the model and should not be tuned to try. ASSUMPTION on a cost-recovery basis.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>⚠ INFERRED - THE WEAKEST OF THE THREE. No GCC platform outside the UAE publishes an average ticket; this is a CONFIRMED NEGATIVE, not a gap in the search. Taken as the UAE figure scaled by the regional income gap (SIP 26.00/33.60 = 0.77x). Do not present this as sourced.</t>
+          <t>INFERRED - THE WEAKEST OF THE THREE. No GCC platform outside the UAE publishes an average ticket; this is a CONFIRMED NEGATIVE, not a gap in the search. Taken as the UAE figure scaled by the regional income gap (SIP 26.00/33.60 = 0.77x). Do not present this as sourced.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>OBSERVED, PROXY. Augmont: average festive-season purchase Rs 3,300, Times of India, Sep 2025 (= ~USD 38). Augmont is a licensed refiner and digital gold platform; a festive lump is structurally the same act as a spot purchase, which is why it is preferred to the alternatives. REJECTED: SafeGold Rs 5,000-8,000 (May 2026) - that book skews to investors, while Aurumix's Indian customer saves USD 30 a month; MMTC-PAMP Rs 800-1,200 - closer to routine micro-saving than a lump; Rs 230 industry-wide - a LinkedIn aggregate, not a citable source. ⚠ WEAKER THAN THE UAE FIGURE: right country and right behaviour, but Aurumix's Indian customer is poorer than Augmont's average buyer, so 40 may be generous.</t>
+          <t>OBSERVED, PROXY. Augmont: average festive-season purchase Rs 3,300, Times of India, Sep 2025 (= ~USD 38). Augmont is a licensed refiner and digital gold platform; a festive lump is structurally the same act as a spot purchase, which is why it is preferred to the alternatives. REJECTED: SafeGold Rs 5,000-8,000 (May 2026) - that book skews to investors, while Aurumix's Indian customer saves USD 30 a month; MMTC-PAMP Rs 800-1,200 - closer to routine micro-saving than a lump; Rs 230 industry-wide - a LinkedIn aggregate, not a citable source. WEAKER THAN THE UAE FIGURE: right country and right behaviour, but Aurumix's Indian customer is poorer than Augmont's average buyer, so 40 may be generous.</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. ⚠ NO PUBLISHED BENCHMARK EXISTS - confirmed negative. ⚠ KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
+          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. NO PUBLISHED BENCHMARK EXISTS - confirmed negative. KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. ⚠ NO PUBLISHED BENCHMARK EXISTS - confirmed negative. ⚠ KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
+          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. NO PUBLISHED BENCHMARK EXISTS - confirmed negative. KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. ⚠ NO PUBLISHED BENCHMARK EXISTS - confirmed negative. ⚠ KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
+          <t>Share of paying customers who make ANY spot purchase in a year - NOT a monthly rate, and NOT how often a buyer buys (that is the separate frequency input). Set on the affordability ratio above: the spot ticket as a multiple of the same customer's monthly SIP. NO PUBLISHED BENCHMARK EXISTS - confirmed negative. KNOWN SIMPLIFICATION: v2.6 applied a TENURE UPLIFT here ('a 3-year account is ~2x as likely to buy spot as a 6-month account') which v3.0 dropped, so this is flat from day one and OVERSTATES SPOT IN THE EARLY YEARS, when nearly every account is young. Restore the uplift in the Phase 5 simulation. ASSUMPTION, structured on an observable driver.</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>RE-CUT 2026-08-20 from 4.20: the outbound bank transfer fee (USD 1.00-2.50) is REMOVED - that is the customer's cost to bear, not Aurumix's. What remains is Sumsub AML re-screening at 1.85 plus operational handling at ~1.35, both of which Aurumix genuinely pays. ⚠ NOT IN THE REVENUE MODEL: redemption is a COST and arrives with the cost build. This row is carried so the driver is documented and the unit rate already agreed. THE FINDING IT CARRIES IS UNCHANGED AND IS THE POINT - VARA Annex 2 III.E.4 forbids charging ANY fee on redemption, verified verbatim at primary source, so the cost is 100% absorbed, no offsetting revenue exists or can exist, and THERE CAN NEVER BE AN EXIT FEE. DERIVED.</t>
+          <t>RE-CUT 2026-08-20 from 4.20: the outbound bank transfer fee (USD 1.00-2.50) is REMOVED - that is the customer's cost to bear, not Aurumix's. What remains is Sumsub AML re-screening at 1.85 plus operational handling at ~1.35, both of which Aurumix genuinely pays. NOT IN THE REVENUE MODEL: redemption is a COST and arrives with the cost build. This row is carried so the driver is documented and the unit rate already agreed. THE FINDING IT CARRIES IS UNCHANGED AND IS THE POINT - VARA Annex 2 III.E.4 forbids charging ANY fee on redemption, verified verbatim at primary source, so the cost is 100% absorbed, no offsetting revenue exists or can exist, and THERE CAN NEVER BE AN EXIT FEE. DERIVED.</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>M1 (client decision 2026-08-20, moved earlier from M13). The India payment route is ASSUMED SOLVED in this model. ⚠ That is a live assumption, not a settled fact - if the route is not solved, this region does not open at all and roughly a quarter of terminal revenue goes with it.</t>
+          <t>M1 (client decision 2026-08-20, moved earlier from M13). The India payment route is ASSUMED SOLVED in this model. That is a live assumption, not a settled fact - if the route is not solved, this region does not open at all and roughly a quarter of terminal revenue goes with it.</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>UPDATED 2026-08-20. UAE-Indian is 4.36m - the Indian consulate's official count at December 2024, also given as 4.3m by the Embassy of India. The brief carried 3.5m, which is roughly a 2021-22 vintage: the community was 3.89m at December 2023 and 4.36m a year later, having doubled from 2.2m over the decade. UAE-other South Asian is 3.46m, the sum of Pakistani 1.90m, Bangladeshi 0.84m, Nepali 0.36m and Sri Lankan 0.36m - the brief's 3.4m was already correct. These are TOTAL RESIDENT NATIONALS including dependants, which is why the economically-active filter below applies. Oman and Bahrain is an expatriate WORKER count. INDIA IS NOT A DEMOGRAPHIC BASE - it is sized BEHAVIOURALLY from gold ETF folios intersected with active digital-gold holders, so its filters are 100%. ⚠ HELD STATIC over the horizon, which is conservative: the UAE Indian community grew ~12% in the single year to Dec 2024.</t>
+          <t>UPDATED 2026-08-20. UAE-Indian is 4.36m - the Indian consulate's official count at December 2024, also given as 4.3m by the Embassy of India. The brief carried 3.5m, which is roughly a 2021-22 vintage: the community was 3.89m at December 2023 and 4.36m a year later, having doubled from 2.2m over the decade. UAE-other South Asian is 3.46m, the sum of Pakistani 1.90m, Bangladeshi 0.84m, Nepali 0.36m and Sri Lankan 0.36m - the brief's 3.4m was already correct. These are TOTAL RESIDENT NATIONALS including dependants, which is why the economically-active filter below applies. Oman and Bahrain is an expatriate WORKER count. INDIA IS NOT A DEMOGRAPHIC BASE - it is sized BEHAVIOURALLY from gold ETF folios intersected with active digital-gold holders, so its filters are 100%. HELD STATIC over the horizon, which is conservative: the UAE Indian community grew ~12% in the single year to Dec 2024.</t>
         </is>
       </c>
       <c r="F74" s="26" t="n">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>~181,150, against the brief's 165,750. ⚠ THE BRIEF'S 'base x ceiling is the invariant' RULE IS DELIBERATELY BROKEN HERE, and the distinction matters: that rule guards against a METHODOLOGICAL re-cut quietly inflating the market by re-tuning filters, which proves nothing. This is not that - it is a DATA CORRECTION. The UAE Indian population really is 4.36m rather than 3.5m, so the addressable market really is larger. Holding the invariant would mean asserting that penetration falls exactly as population rises, which has no basis. The penetration ceilings are untouched.</t>
+          <t>~181,150, against the brief's 165,750. THE BRIEF'S 'base x ceiling is the invariant' RULE IS DELIBERATELY BROKEN HERE, and the distinction matters: that rule guards against a METHODOLOGICAL re-cut quietly inflating the market by re-tuning filters, which proves nothing. This is not that - it is a DATA CORRECTION. The UAE Indian population really is 4.36m rather than 3.5m, so the addressable market really is larger. Holding the invariant would mean asserting that penetration falls exactly as population rises, which has no basis. The penetration ceilings are untouched.</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>⚠ LIVE, SO IT MOVES IF ANYONE RAISES A CEILING - which is the point. Two INDEPENDENT methods landing within ~2x is the strongest defence of the funnel in this model: the funnel says the UAE can reach ~113,000 SIP accounts, and a real UAE gold app in the same segment has ~75,000 active users today. Our addressable base of ~1.43m sits against 775,000 who explored that product - same order again. If this multiple drifts far above ~2x, the ceiling has stopped being defensible by evidence and is being set by the answer someone wanted. DERIVED from a cited observation.</t>
+          <t>LIVE, SO IT MOVES IF ANYONE RAISES A CEILING - which is the point. Two INDEPENDENT methods landing within ~2x is the strongest defence of the funnel in this model: the funnel says the UAE can reach ~113,000 SIP accounts, and a real UAE gold app in the same segment has ~75,000 active users today. Our addressable base of ~1.43m sits against 775,000 who explored that product - same order again. If this multiple drifts far above ~2x, the ceiling has stopped being defensible by evidence and is being set by the answer someone wanted. DERIVED from a cited observation.</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CONFIRMED NEGATIVE, recorded so it is not re-searched. No GCC platform outside the UAE publishes a user count. India publishes only REGISTERED counts (Jar 35m, Augmont 42m) which cannot be deduplicated or converted to active users, so no comparable cross-check can be built. ⚠ NOTE THAT INDIA'S OWN BASE IS ALREADY user-derived - its 12.5m is 'holds a gold ETF folio or actively buys digital gold', which is why its three filters all sit at 1.00 - AND IT IS THE LEAST TRACEABLE BASE IN THE MODEL. That is the evidence that a user-based method does not automatically produce a better-sourced number.</t>
+          <t>CONFIRMED NEGATIVE, recorded so it is not re-searched. No GCC platform outside the UAE publishes a user count. India publishes only REGISTERED counts (Jar 35m, Augmont 42m) which cannot be deduplicated or converted to active users, so no comparable cross-check can be built. NOTE THAT INDIA'S OWN BASE IS ALREADY user-derived - its 12.5m is 'holds a gold ETF folio or actively buys digital gold', which is why its three filters all sit at 1.00 - AND IT IS THE LEAST TRACEABLE BASE IN THE MODEL. That is the evidence that a user-based method does not automatically produce a better-sourced number.</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. ⚠ COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. ⚠ AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
+          <t>RAISED 50% on 2026-08-21. A STOCK, NOT A FLOW: at 45% attrition, holding 186 active needs ~84 recruits a year just to stand still, and reaching 186 from 8 means recruiting and training several hundred people over seven years. COMPOUNDS WITH AGENT PRODUCTIVITY, raised from 4 to 6 the same day - together they are 2.25x the agent output the model carried this morning. AND IT IS A COST THIS MODEL CANNOT SEE: agents are paid, and the salesforce is now 45% UAE / 10% Oman &amp; Bahrain / 45% India, where a Dubai salesperson and an Indian commission agent are not remotely the same expense. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. 🔴 THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. ⚠ IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
+          <t>RAISED 50% on 2026-08-21, client instruction. A DECISION VARIABLE and an input to acquisition, not an output of a cost table. THE SINGLE LARGEST LEVER IN THE MODEL AND THE ONLY ONE THAT IS PURELY A SPENDING CHOICE: measured sensitivity puts +50% here at +28.5% customers and +29.3% gold. IT IS ALSO THE ONE THE REVENUE-ONLY SCOPE FLATTERS MOST. This model has no cost side yet, so an extra USD 1.9m of marketing across the horizon appears here as pure upside. It is not - it is USD 1.9m of spend, and whether it is worth making is a question only the cost build can answer. DO NOT PRESENT THE UPLIFT FROM THIS ROW AS PROFIT.</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. ⚠ IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. ⚠ NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
+          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. ⚠ IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. ⚠ NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
+          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3195,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. ⚠ IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. ⚠ NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
+          <t>REVISED 2026-08-20. An earlier cut put 100% in India, which left the UAE - the licensed home market - with no people selling at all. There will be a salesforce outside India; it is simply SALARIED rather than commission-only. FOR REVENUE THE DISTINCTION DOES NOT MATTER: both are people acquiring customers at some productivity. IT MATTERS ENORMOUSLY FOR COST - a Dubai salesperson and an Indian commission agent are not remotely the same expense, and this split MUST be cost-weighted when the cost build lands. India stays high because a large agent pool is cheapest to build there; UAE is weighted for being the core licensed market. NOT the same thing as stream 6: that is B2B, partners white-labelling the platform onto their own customer books, and is not a consumer sales channel at all. Must sum to 100%. CLIENT INPUT.</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ADDED 2026-08-21, client instruction, replacing a flat price. 8.1% is the COMPOUND ANNUAL GROWTH RATE SINCE 1971, the end of the gold standard - chosen because it is the LONGEST window and therefore the least cherry-picked. The shorter the window the better gold looks: ~8.6% over 50 years, ~9-10% over 20, ~13-14% over 10, and over 20% over the last 5. Taking the recent decade would have flattered the model on a rally. CITED. ⚠ THIS IS A NOMINAL RATE AND NOTHING ELSE IN THE MODEL INFLATES. SIP tickets, spot tickets, CAC, card fees and the B2B fee are all frozen in 2027 dollars. There is NO CONSENSUS POSITIVE LONG-RUN REAL RETURN for gold - it is generally treated as a store of value with a near-zero real yield - so most of this 8.1% IS INFLATION. Applying it to the metal while freezing everything else quietly asserts that gold outruns wages, prices and costs by 8% a year for seven years, which is not a claim anyone would defend out loud. The Model therefore also carries AUM AT THE CONSTANT M1 PRICE, and that is the honest series for judging whether the BUSINESS grew. Conservative is set at 0.0% deliberately: it restores the original flat-price design, under which every revenue change is attributable to the business rather than the metal.</t>
+          <t>ADDED 2026-08-21, client instruction, replacing a flat price. 8.1% is the COMPOUND ANNUAL GROWTH RATE SINCE 1971, the end of the gold standard - chosen because it is the LONGEST window and therefore the least cherry-picked. The shorter the window the better gold looks: ~8.6% over 50 years, ~9-10% over 20, ~13-14% over 10, and over 20% over the last 5. Taking the recent decade would have flattered the model on a rally. CITED. THIS IS A NOMINAL RATE AND NOTHING ELSE IN THE MODEL INFLATES. SIP tickets, spot tickets, CAC, card fees and the B2B fee are all frozen in 2027 dollars. There is NO CONSENSUS POSITIVE LONG-RUN REAL RETURN for gold - it is generally treated as a store of value with a near-zero real yield - so most of this 8.1% IS INFLATION. Applying it to the metal while freezing everything else quietly asserts that gold outruns wages, prices and costs by 8% a year for seven years, which is not a claim anyone would defend out loud. The Model therefore also carries AUM AT THE CONSTANT M1 PRICE, and that is the honest series for judging whether the BUSINESS grew. Conservative is set at 0.0% deliberately: it restores the original flat-price design, under which every revenue change is attributable to the business rather than the metal.</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 4, client instruction. The insurance agency comparator that produced 4 is for agents selling a COMPLEX UNDERWRITTEN PRODUCT with medical questions and multi-page forms; a gold SIP signup is a fraction of that work, so the comparator was conservative for this product. ⚠ COMPOUNDS WITH THE AGENT HEADCOUNT, which was raised 50% the same day - together they are 2.25x the agent output the model carried this morning. Both are execution assumptions with no external anchor at the new level; if either disappoints, the other does not compensate. TRIANGULATED at 4, ASSUMPTION at 6.</t>
+          <t>RAISED 2026-08-21 from 4, client instruction. The insurance agency comparator that produced 4 is for agents selling a COMPLEX UNDERWRITTEN PRODUCT with medical questions and multi-page forms; a gold SIP signup is a fraction of that work, so the comparator was conservative for this product. COMPOUNDS WITH THE AGENT HEADCOUNT, which was raised 50% the same day - together they are 2.25x the agent output the model carried this morning. Both are execution assumptions with no external anchor at the new level; if either disappoints, the other does not compensate. TRIANGULATED at 4, ASSUMPTION at 6.</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 0.45, client instruction. Cap removed deliberately, so the distribution is right-skewed - MODEL THE MEAN, NOT THE MEDIAN. 0.60 means the average customer produces roughly three referrals every five years; the mean is pulled up by a small number of highly social referrers, which is the normal shape for a trust-based product inside a tight diaspora community. ⚠ IT IS STILL AN ASSUMPTION WITH NO EXTERNAL ANCHOR, and it compounds: referrals feed the paying base, which feeds more referrals. That loop is the reason this parameter is more load-bearing than its size suggests. ASSUMPTION.</t>
+          <t>RAISED 2026-08-21 from 0.45, client instruction. Cap removed deliberately, so the distribution is right-skewed - MODEL THE MEAN, NOT THE MEDIAN. 0.60 means the average customer produces roughly three referrals every five years; the mean is pulled up by a small number of highly social referrers, which is the normal shape for a trust-based product inside a tight diaspora community. IT IS STILL AN ASSUMPTION WITH NO EXTERNAL ANCHOR, and it compounds: referrals feed the paying base, which feeds more referrals. That loop is the reason this parameter is more load-bearing than its size suggests. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 0.12, client instruction. Kept separate from CAC deliberately, so the acquisition cost never applies to it - THAT IS ALSO WHY IT IS AN ATTRACTIVE NUMBER TO RAISE, and why it deserves scepticism. 0.25 says a quarter of paid-driven signups arrive again for free through word of mouth, app store discovery and community effects. Defensible for a product sold inside a dense diaspora network where the paid campaign and the community overlap almost completely. ⚠ NO EXTERNAL ANCHOR AT EITHER LEVEL, and it is arithmetically identical to a 12% CAC reduction - so raising this AND cutting CAC in the same pass is close to taking the same benefit twice. ASSUMPTION.</t>
+          <t>RAISED 2026-08-21 from 0.12, client instruction. Kept separate from CAC deliberately, so the acquisition cost never applies to it - THAT IS ALSO WHY IT IS AN ATTRACTIVE NUMBER TO RAISE, and why it deserves scepticism. 0.25 says a quarter of paid-driven signups arrive again for free through word of mouth, app store discovery and community effects. Defensible for a product sold inside a dense diaspora network where the paid campaign and the community overlap almost completely. NO EXTERNAL ANCHOR AT EITHER LEVEL, and it is arithmetically identical to a 12% CAC reduction - so raising this AND cutting CAC in the same pass is close to taking the same benefit twice. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>HALVED 2026-08-21 from 0.12, client instruction. ⚠ NOTE IT HAS ZERO EFFECT ON GOLD UNDER CUSTODY - measured, not asserted - because self-custodied metal never left the vault and was never in that measure. It moves ONLY the collateral-eligible base and therefore the card credit limit, worth ~0.2% of Y7 revenue. RELABELLED earlier the same day after the client correctly objected to the old name, 'self-custody leakage'. THE GOLD DOES NOT LEAVE THE VAULT: a token moving to a customer's own wallet sells nothing and burns nothing, so calling it an AUM decrease was wrong. What it does leave is Aurumix's COLLATERAL-ELIGIBLE base - Aurumix cannot foreclose on a token sitting in a private wallet, so that gold can no longer back a credit limit. In this model AUM has exactly ONE consumer, the card credit limit, so the arithmetic was always right and only the label was misleading. ⚠ THAT ONE-CONSUMER PROPERTY IS WHAT MAKES THIS SAFE: if a later build points anything else at AUM - a custody fee, a reported-AUM headline - this row must be split in two first. Contrast the redemption line, which IS gold genuinely gone. ASSUMPTION.</t>
+          <t>HALVED 2026-08-21 from 0.12, client instruction. NOTE IT HAS ZERO EFFECT ON GOLD UNDER CUSTODY - measured, not asserted - because self-custodied metal never left the vault and was never in that measure. It moves ONLY the collateral-eligible base and therefore the card credit limit, worth ~0.2% of Y7 revenue. RELABELLED earlier the same day after the client correctly objected to the old name, 'self-custody leakage'. THE GOLD DOES NOT LEAVE THE VAULT: a token moving to a customer's own wallet sells nothing and burns nothing, so calling it an AUM decrease was wrong. What it does leave is Aurumix's COLLATERAL-ELIGIBLE base - Aurumix cannot foreclose on a token sitting in a private wallet, so that gold can no longer back a credit limit. In this model AUM has exactly ONE consumer, the card credit limit, so the arithmetic was always right and only the label was misleading. THAT ONE-CONSUMER PROPERTY IS WHAT MAKES THIS SAFE: if a later build points anything else at AUM - a custody fee, a reported-AUM headline - this row must be split in two first. Contrast the redemption line, which IS gold genuinely gone. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>LOWERED 2026-08-21 from 2.2, client instruction. ⚠ THIS IS THE WEAKEST OF THE THREE DECAY CHANGES. The LOGIC behind a multiplier above 1.0 is untouched and still holds: customers who stopped paying redeem faster, because they have no accruing benefit left to protect. Lowering it to 1.6 weakens that argument without new evidence for the smaller number - it says lapsed customers are stickier than previously assumed, which is the convenient direction. Because holders become the majority of the book by Y4, this remains the DOMINANT AUM DECAY TERM from roughly Y4, so the change is not cosmetic. ASSUMPTION, and the first one to revisit if AUM is challenged.</t>
+          <t>LOWERED 2026-08-21 from 2.2, client instruction. THIS IS THE WEAKEST OF THE THREE DECAY CHANGES. The LOGIC behind a multiplier above 1.0 is untouched and still holds: customers who stopped paying redeem faster, because they have no accruing benefit left to protect. Lowering it to 1.6 weakens that argument without new evidence for the smaller number - it says lapsed customers are stickier than previously assumed, which is the convenient direction. Because holders become the majority of the book by Y4, this remains the DOMINANT AUM DECAY TERM from roughly Y4, so the change is not cosmetic. ASSUMPTION, and the first one to revisit if AUM is challenged.</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>REPLACED the global 'Average spot ticket' on 2026-08-21. The LEVEL is no longer a scenario input: each region now carries its own OBSERVED ticket on Assumptions (UAE 190 from Botim, India 40 from Augmont, Oman &amp; Bahrain 145 inferred). This parameter carries only the UNCERTAINTY around those observations, as a single dial. ⚠ WHY ONE DIAL AND NOT THREE: three regional triplets would be nine numbers to defend and would let a scenario silently invert the regional ordering that the sources establish. One multiplier flexes the level and PRESERVES the ordering. Aggressive 1.35 puts the UAE at ~257, still under the AED 1,000 mark; conservative 0.70 puts it at ~133, below Botim's own sub-AED-500 majority. ASSUMPTION about spread, applied to observed levels.</t>
+          <t>REPLACED the global 'Average spot ticket' on 2026-08-21. The LEVEL is no longer a scenario input: each region now carries its own OBSERVED ticket on Assumptions (UAE 190 from Botim, India 40 from Augmont, Oman &amp; Bahrain 145 inferred). This parameter carries only the UNCERTAINTY around those observations, as a single dial. WHY ONE DIAL AND NOT THREE: three regional triplets would be nine numbers to defend and would let a scenario silently invert the regional ordering that the sources establish. One multiplier flexes the level and PRESERVES the ordering. Aggressive 1.35 puts the UAE at ~257, still under the AED 1,000 mark; conservative 0.70 puts it at ~133, below Botim's own sub-AED-500 majority. ASSUMPTION about spread, applied to observed levels.</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>⚠ PROVENANCE CORRECTED 2026-08-21 - THE NUMBER STANDS, ITS OLD CITATION DID NOT. The previous note read 'Botim's 128,000 trades against ~45,000 buyers implies ~1.9/yr'. THE 45,000 IS NOT A BUYER COUNT, IT IS A TRANSACTION COUNT: Khaleej Times, Nov 2025, says 775,000 users EXPLORED the feature, 'completing over 45,000 transactions'. The 128,000 is also transactions, to Feb 2026. So the old derivation divided transactions by transactions across two different windows - the result was the growth in cumulative trades, not a frequency. CONFIRMED NEGATIVE: Botim has never published a unique-buyer count, so no frequency can be derived from it, and no published frequency exists ANYWHERE for ad-hoc lump gold purchases. Comparators are 0.85/yr (Augmont, per REGISTERED user, at an average transaction of Rs 331 - micro-saving, not lumps) and 264/yr (Jar, Rs 10/day auto-roundups) - a 300x spread, neither being this product. WHAT DOES SUPPORT 1.7 is a cross-check on the COMBINED basis, attach x frequency x ticket, which is comparable: Aurumix India implies ~Rs 838/yr of gold per paying customer against Augmont's ~Rs 281/yr per registered user. 3x, and defensible - our customers are engaged SIP savers, not dormant registrations. Behaviourally 1.7 is also about right for festive lumps: Dhanteras, Akshaya Tritiya and a wedding is roughly two events. ASSUMPTION, cross-checked on the combined basis, NOT directly sourced.</t>
+          <t>PROVENANCE CORRECTED 2026-08-21 - THE NUMBER STANDS, ITS OLD CITATION DID NOT. The previous note read 'Botim's 128,000 trades against ~45,000 buyers implies ~1.9/yr'. THE 45,000 IS NOT A BUYER COUNT, IT IS A TRANSACTION COUNT: Khaleej Times, Nov 2025, says 775,000 users EXPLORED the feature, 'completing over 45,000 transactions'. The 128,000 is also transactions, to Feb 2026. So the old derivation divided transactions by transactions across two different windows - the result was the growth in cumulative trades, not a frequency. CONFIRMED NEGATIVE: Botim has never published a unique-buyer count, so no frequency can be derived from it, and no published frequency exists ANYWHERE for ad-hoc lump gold purchases. Comparators are 0.85/yr (Augmont, per REGISTERED user, at an average transaction of Rs 331 - micro-saving, not lumps) and 264/yr (Jar, Rs 10/day auto-roundups) - a 300x spread, neither being this product. WHAT DOES SUPPORT 1.7 is a cross-check on the COMBINED basis, attach x frequency x ticket, which is comparable: Aurumix India implies ~Rs 838/yr of gold per paying customer against Augmont's ~Rs 281/yr per registered user. 3x, and defensible - our customers are engaged SIP savers, not dormant registrations. Behaviourally 1.7 is also about right for festive lumps: Dhanteras, Akshaya Tritiya and a wedding is roughly two events. ASSUMPTION, cross-checked on the combined basis, NOT directly sourced.</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-20, client decision: THE CARD IS A DRAWDOWN ON THE GOLD-COLLATERALISED FACILITY, not a salary-repaid revolving card. Aurumix has no balance sheet to lend from - it can only extend credit against collateral it holds, which is the customer's gold. Using the card IS borrowing, so card activation and credit take-up are the SAME behaviour and were previously modelled as two different populations (50% activating a card, 18% taking credit) doing what is in fact one thing. Merged onto the credit figure, which is the better-anchored of the two: Indian gold-loan penetration is under 10% at a point in time, uplifted here for pre-selection since these customers have already cleared a six-payment gate. ⚠ THE OLD 50% CAME FROM NEOBANK COMPARABLES (PULSE 68.2%, Monzo 68%) WHERE THE CARD IS THE PRODUCT - wrong in kind for a card that only lets you borrow against your own savings. DERIVED.</t>
+          <t>RE-BASED 2026-08-20, client decision: THE CARD IS A DRAWDOWN ON THE GOLD-COLLATERALISED FACILITY, not a salary-repaid revolving card. Aurumix has no balance sheet to lend from - it can only extend credit against collateral it holds, which is the customer's gold. Using the card IS borrowing, so card activation and credit take-up are the SAME behaviour and were previously modelled as two different populations (50% activating a card, 18% taking credit) doing what is in fact one thing. Merged onto the credit figure, which is the better-anchored of the two: Indian gold-loan penetration is under 10% at a point in time, uplifted here for pre-selection since these customers have already cleared a six-payment gate. THE OLD 50% CAME FROM NEOBANK COMPARABLES (PULSE 68.2%, Monzo 68%) WHERE THE CARD IS THE PRODUCT - wrong in kind for a card that only lets you borrow against your own savings. DERIVED.</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-20 from 12 transactions/MONTH once the card became a drawdown on the gold facility. Under that model the customer borrows a lump (limit x drawn share) a couple of times a year and spends it down, so the meaningful unit is transactions PER DRAW, not per month. At 12/month the implied ticket collapsed to ~AED 12, which is a coffee, not a reason to pledge your gold. THE AVERAGE TICKET FALLS OUT AS drawn amount / this number, and the draw events cancel - so the ticket depends only on how large a draw is and how many purchases it is spent across. ⚠ IT ALSO CHANGES WHAT THE CARD IS FOR: not daily groceries, but occasional larger needs - school fees, a medical bill, an emergency - funded by borrowing against savings rather than liquidating them. That is a materially different product story and should be put to the client in those words. ASSUMPTION.</t>
+          <t>RE-BASED 2026-08-20 from 12 transactions/MONTH once the card became a drawdown on the gold facility. Under that model the customer borrows a lump (limit x drawn share) a couple of times a year and spends it down, so the meaningful unit is transactions PER DRAW, not per month. At 12/month the implied ticket collapsed to ~AED 12, which is a coffee, not a reason to pledge your gold. THE AVERAGE TICKET FALLS OUT AS drawn amount / this number, and the draw events cancel - so the ticket depends only on how large a draw is and how many purchases it is spent across. IT ALSO CHANGES WHAT THE CARD IS FOR: not daily groceries, but occasional larger needs - school fees, a medical bill, an emergency - funded by borrowing against savings rather than liquidating them. That is a materially different product story and should be put to the client in those words. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>SET AT 0.15 on 2026-08-21, client instruction - the same day it came DOWN from 0.20 to 0.08, so it has landed close to where it started. What has genuinely changed is not the number but the STRUCTURE. ⚠ THE UNIT ALSO CHANGED, AND THAT MATTERS: it is now the share of NEW customers who take the plan when they join, feeding a SUBSCRIBER BALANCE that then churns - not a standing share of the whole book that could never fall. The steady-state share of paying customers holding a plan therefore lands BELOW this number. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on; 20% is at the top of the normal range for an OPTIONAL PAID extra on a savings product, which is low single digits to low teens. ⚠ IT IS NOT EQUIVALENT TO THE OLD 20% AND SHOULD NOT BE READ AS A PARTIAL REVERSAL: 20% was a permanent share of the whole book that could never decay, while 15% applies once, on joining, to a balance that then churns at ~7.1% a month. The standing share of paying customers holding a plan settles near 10.5%, not 15%. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on. ASSUMPTION.</t>
+          <t>SET AT 0.15 on 2026-08-21, client instruction - the same day it came DOWN from 0.20 to 0.08, so it has landed close to where it started. What has genuinely changed is not the number but the STRUCTURE. THE UNIT ALSO CHANGED, AND THAT MATTERS: it is now the share of NEW customers who take the plan when they join, feeding a SUBSCRIBER BALANCE that then churns - not a standing share of the whole book that could never fall. The steady-state share of paying customers holding a plan therefore lands BELOW this number. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on; 20% is at the top of the normal range for an OPTIONAL PAID extra on a savings product, which is low single digits to low teens. IT IS NOT EQUIVALENT TO THE OLD 20% AND SHOULD NOT BE READ AS A PARTIAL REVERSAL: 20% was a permanent share of the whole book that could never decay, while 15% applies once, on joining, to a balance that then churns at ~7.1% a month. The standing share of paying customers holding a plan settles near 10.5%, not 15%. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>ADDED 2026-08-21. THE FIRST IS INCLUDED IN THE PLAN PRICE, so only the excess over 1.0 is charged - at 2.5 that is 1.5 chargeable. No platform publishes beneficiaries-per-will. What anchors it is who these customers are: South Asian migrant workers who remit ~80% of income to families at home, typically supporting a spouse, children and parents. Household sizes in the source countries run ~4.4 in India, ~4.5 in Bangladesh and ~6.8 in Pakistan, so naming 2-3 beneficiaries is conservative against the family they actually support. ⚠ NOT THE SAME AS HOUSEHOLD SIZE - a beneficiary is a named, identity-verified person on a legal instrument, and people name fewer than they support. ASSUMPTION anchored on demographics.</t>
+          <t>ADDED 2026-08-21. THE FIRST IS INCLUDED IN THE PLAN PRICE, so only the excess over 1.0 is charged - at 2.5 that is 1.5 chargeable. No platform publishes beneficiaries-per-will. What anchors it is who these customers are: South Asian migrant workers who remit ~80% of income to families at home, typically supporting a spouse, children and parents. Household sizes in the source countries run ~4.4 in India, ~4.5 in Bangladesh and ~6.8 in Pakistan, so naming 2-3 beneficiaries is conservative against the family they actually support. NOT THE SAME AS HOUSEHOLD SIZE - a beneficiary is a named, identity-verified person on a legal instrument, and people name fewer than they support. ASSUMPTION anchored on demographics.</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>THE MIX, NOT THE BIGGEST. A realistic six-partner Gulf book is roughly one Botim-scale (1.7m ACTIVE fintech users, of 8.2-8.5m app users), two at e&amp; money scale (~1.5m subscribers), and three small wallets at a few hundred thousand - which averages near 900k. ⚠ USE ACTIVE USERS, NOT REGISTERED: Botim's own numbers separate 8.5m app users, 3m KYC'd and 1.7m active fintech users, and adopting the headline would overstate this by 5x. CITED for the two largest, ASSUMPTION for the tail.</t>
+          <t>THE MIX, NOT THE BIGGEST. A realistic six-partner Gulf book is roughly one Botim-scale (1.7m ACTIVE fintech users, of 8.2-8.5m app users), two at e&amp; money scale (~1.5m subscribers), and three small wallets at a few hundred thousand - which averages near 900k. USE ACTIVE USERS, NOT REGISTERED: Botim's own numbers separate 8.5m app users, 3m KYC'd and 1.7m active fintech users, and adopting the headline would overstate this by 5x. CITED for the two largest, ASSUMPTION for the tail.</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>OBSERVED ANCHOR: O Gold reports 75,000 ACTIVE users against Botim's 1.7m active fintech users - 4.4% - and 775,000 who merely explored the feature. Base is set at 6%, ABOVE the observed 4.4%, because that figure is roughly six months after the gold feature launched and adoption should mature; 6% is a 1.4x maturation, not a doubling. ⚠ THE 4.4% IS THE ONLY OBSERVED GOLD-ADOPTION RATE FOR A GULF WALLET THAT EXISTS. TRIANGULATED.</t>
+          <t>OBSERVED ANCHOR: O Gold reports 75,000 ACTIVE users against Botim's 1.7m active fintech users - 4.4% - and 775,000 who merely explored the feature. Base is set at 6%, ABOVE the observed 4.4%, because that figure is roughly six months after the gold feature launched and adoption should mature; 6% is a 1.4x maturation, not a doubling. THE 4.4% IS THE ONLY OBSERVED GOLD-ADOPTION RATE FOR A GULF WALLET THAT EXISTS. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>ADDED 2026-08-21, client instruction, replacing a flat price. 8.1% is the COMPOUND ANNUAL GROWTH RATE SINCE 1971, the end of the gold standard - chosen because it is the LONGEST window and therefore the least cherry-picked. The shorter the window the better gold looks: ~8.6% over 50 years, ~9-10% over 20, ~13-14% over 10, and over 20% over the last 5. Taking the recent decade would have flattered the model on a rally. CITED. ⚠ THIS IS A NOMINAL RATE AND NOTHING ELSE IN THE MODEL INFLATES. SIP tickets, spot tickets, CAC, card fees and the B2B fee are all frozen in 2027 dollars. There is NO CONSENSUS POSITIVE LONG-RUN REAL RETURN for gold - it is generally treated as a store of value with a near-zero real yield - so most of this 8.1% IS INFLATION. Applying it to the metal while freezing everything else quietly asserts that gold outruns wages, prices and costs by 8% a year for seven years, which is not a claim anyone would defend out loud. The Model therefore also carries AUM AT THE CONSTANT M1 PRICE, and that is the honest series for judging whether the BUSINESS grew. Conservative is set at 0.0% deliberately: it restores the original flat-price design, under which every revenue change is attributable to the business rather than the metal.</t>
+          <t>ADDED 2026-08-21, client instruction, replacing a flat price. 8.1% is the COMPOUND ANNUAL GROWTH RATE SINCE 1971, the end of the gold standard - chosen because it is the LONGEST window and therefore the least cherry-picked. The shorter the window the better gold looks: ~8.6% over 50 years, ~9-10% over 20, ~13-14% over 10, and over 20% over the last 5. Taking the recent decade would have flattered the model on a rally. CITED. THIS IS A NOMINAL RATE AND NOTHING ELSE IN THE MODEL INFLATES. SIP tickets, spot tickets, CAC, card fees and the B2B fee are all frozen in 2027 dollars. There is NO CONSENSUS POSITIVE LONG-RUN REAL RETURN for gold - it is generally treated as a store of value with a near-zero real yield - so most of this 8.1% IS INFLATION. Applying it to the metal while freezing everything else quietly asserts that gold outruns wages, prices and costs by 8% a year for seven years, which is not a claim anyone would defend out loud. The Model therefore also carries AUM AT THE CONSTANT M1 PRICE, and that is the honest series for judging whether the BUSINESS grew. Conservative is set at 0.0% deliberately: it restores the original flat-price design, under which every revenue change is attributable to the business rather than the metal.</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 4, client instruction. The insurance agency comparator that produced 4 is for agents selling a COMPLEX UNDERWRITTEN PRODUCT with medical questions and multi-page forms; a gold SIP signup is a fraction of that work, so the comparator was conservative for this product. ⚠ COMPOUNDS WITH THE AGENT HEADCOUNT, which was raised 50% the same day - together they are 2.25x the agent output the model carried this morning. Both are execution assumptions with no external anchor at the new level; if either disappoints, the other does not compensate. TRIANGULATED at 4, ASSUMPTION at 6.</t>
+          <t>RAISED 2026-08-21 from 4, client instruction. The insurance agency comparator that produced 4 is for agents selling a COMPLEX UNDERWRITTEN PRODUCT with medical questions and multi-page forms; a gold SIP signup is a fraction of that work, so the comparator was conservative for this product. COMPOUNDS WITH THE AGENT HEADCOUNT, which was raised 50% the same day - together they are 2.25x the agent output the model carried this morning. Both are execution assumptions with no external anchor at the new level; if either disappoints, the other does not compensate. TRIANGULATED at 4, ASSUMPTION at 6.</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; ⚠ note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
+          <t>REGIONALISED 2026-08-20. A single global USD 120 was applied everywhere, which is roughly right for the UAE and badly wrong for India. PUBLISHED BENCHMARKS: Dubai consumer fintech USD 65-220; retail neobank account paid-only USD 35-70; GCC wealthtech funded accounts USD 80-220; 'true' fully-loaded CAC per ACTIVATED customer USD 85-350 against USD 50-100 reported, once KYC, onboarding and non-activating signups are counted. INDIA IS A DIFFERENT MARKET ENTIRELY: consumer fintech INR 500-1,500 (~USD 6-18), neobank savings activation INR 1,100-1,800, wealth and broking apps INR 2,500-5,500 (~USD 30-65); Jupiter reports a USD 5-6 paid CAC. USD 120 is ~INR 10,500 - some 7-20x the Indian mass-market benchmark and still 2-4x its premium wealth apps. UAE is held at 120 as a FULLY-LOADED figure; note it sits at the top of the range for a LOW-TICKET product, and the published low-ticket band is USD 4-70. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 0.45, client instruction. Cap removed deliberately, so the distribution is right-skewed - MODEL THE MEAN, NOT THE MEDIAN. 0.60 means the average customer produces roughly three referrals every five years; the mean is pulled up by a small number of highly social referrers, which is the normal shape for a trust-based product inside a tight diaspora community. ⚠ IT IS STILL AN ASSUMPTION WITH NO EXTERNAL ANCHOR, and it compounds: referrals feed the paying base, which feeds more referrals. That loop is the reason this parameter is more load-bearing than its size suggests. ASSUMPTION.</t>
+          <t>RAISED 2026-08-21 from 0.45, client instruction. Cap removed deliberately, so the distribution is right-skewed - MODEL THE MEAN, NOT THE MEDIAN. 0.60 means the average customer produces roughly three referrals every five years; the mean is pulled up by a small number of highly social referrers, which is the normal shape for a trust-based product inside a tight diaspora community. IT IS STILL AN ASSUMPTION WITH NO EXTERNAL ANCHOR, and it compounds: referrals feed the paying base, which feeds more referrals. That loop is the reason this parameter is more load-bearing than its size suggests. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21 from 0.12, client instruction. Kept separate from CAC deliberately, so the acquisition cost never applies to it - THAT IS ALSO WHY IT IS AN ATTRACTIVE NUMBER TO RAISE, and why it deserves scepticism. 0.25 says a quarter of paid-driven signups arrive again for free through word of mouth, app store discovery and community effects. Defensible for a product sold inside a dense diaspora network where the paid campaign and the community overlap almost completely. ⚠ NO EXTERNAL ANCHOR AT EITHER LEVEL, and it is arithmetically identical to a 12% CAC reduction - so raising this AND cutting CAC in the same pass is close to taking the same benefit twice. ASSUMPTION.</t>
+          <t>RAISED 2026-08-21 from 0.12, client instruction. Kept separate from CAC deliberately, so the acquisition cost never applies to it - THAT IS ALSO WHY IT IS AN ATTRACTIVE NUMBER TO RAISE, and why it deserves scepticism. 0.25 says a quarter of paid-driven signups arrive again for free through word of mouth, app store discovery and community effects. Defensible for a product sold inside a dense diaspora network where the paid campaign and the community overlap almost completely. NO EXTERNAL ANCHOR AT EITHER LEVEL, and it is arithmetically identical to a 12% CAC reduction - so raising this AND cutting CAC in the same pass is close to taking the same benefit twice. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>HALVED 2026-08-21 from 0.12, client instruction. ⚠ NOTE IT HAS ZERO EFFECT ON GOLD UNDER CUSTODY - measured, not asserted - because self-custodied metal never left the vault and was never in that measure. It moves ONLY the collateral-eligible base and therefore the card credit limit, worth ~0.2% of Y7 revenue. RELABELLED earlier the same day after the client correctly objected to the old name, 'self-custody leakage'. THE GOLD DOES NOT LEAVE THE VAULT: a token moving to a customer's own wallet sells nothing and burns nothing, so calling it an AUM decrease was wrong. What it does leave is Aurumix's COLLATERAL-ELIGIBLE base - Aurumix cannot foreclose on a token sitting in a private wallet, so that gold can no longer back a credit limit. In this model AUM has exactly ONE consumer, the card credit limit, so the arithmetic was always right and only the label was misleading. ⚠ THAT ONE-CONSUMER PROPERTY IS WHAT MAKES THIS SAFE: if a later build points anything else at AUM - a custody fee, a reported-AUM headline - this row must be split in two first. Contrast the redemption line, which IS gold genuinely gone. ASSUMPTION.</t>
+          <t>HALVED 2026-08-21 from 0.12, client instruction. NOTE IT HAS ZERO EFFECT ON GOLD UNDER CUSTODY - measured, not asserted - because self-custodied metal never left the vault and was never in that measure. It moves ONLY the collateral-eligible base and therefore the card credit limit, worth ~0.2% of Y7 revenue. RELABELLED earlier the same day after the client correctly objected to the old name, 'self-custody leakage'. THE GOLD DOES NOT LEAVE THE VAULT: a token moving to a customer's own wallet sells nothing and burns nothing, so calling it an AUM decrease was wrong. What it does leave is Aurumix's COLLATERAL-ELIGIBLE base - Aurumix cannot foreclose on a token sitting in a private wallet, so that gold can no longer back a credit limit. In this model AUM has exactly ONE consumer, the card credit limit, so the arithmetic was always right and only the label was misleading. THAT ONE-CONSUMER PROPERTY IS WHAT MAKES THIS SAFE: if a later build points anything else at AUM - a custody fee, a reported-AUM headline - this row must be split in two first. Contrast the redemption line, which IS gold genuinely gone. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>LOWERED 2026-08-21 from 2.2, client instruction. ⚠ THIS IS THE WEAKEST OF THE THREE DECAY CHANGES. The LOGIC behind a multiplier above 1.0 is untouched and still holds: customers who stopped paying redeem faster, because they have no accruing benefit left to protect. Lowering it to 1.6 weakens that argument without new evidence for the smaller number - it says lapsed customers are stickier than previously assumed, which is the convenient direction. Because holders become the majority of the book by Y4, this remains the DOMINANT AUM DECAY TERM from roughly Y4, so the change is not cosmetic. ASSUMPTION, and the first one to revisit if AUM is challenged.</t>
+          <t>LOWERED 2026-08-21 from 2.2, client instruction. THIS IS THE WEAKEST OF THE THREE DECAY CHANGES. The LOGIC behind a multiplier above 1.0 is untouched and still holds: customers who stopped paying redeem faster, because they have no accruing benefit left to protect. Lowering it to 1.6 weakens that argument without new evidence for the smaller number - it says lapsed customers are stickier than previously assumed, which is the convenient direction. Because holders become the majority of the book by Y4, this remains the DOMINANT AUM DECAY TERM from roughly Y4, so the change is not cosmetic. ASSUMPTION, and the first one to revisit if AUM is challenged.</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>REPLACED the global 'Average spot ticket' on 2026-08-21. The LEVEL is no longer a scenario input: each region now carries its own OBSERVED ticket on Assumptions (UAE 190 from Botim, India 40 from Augmont, Oman &amp; Bahrain 145 inferred). This parameter carries only the UNCERTAINTY around those observations, as a single dial. ⚠ WHY ONE DIAL AND NOT THREE: three regional triplets would be nine numbers to defend and would let a scenario silently invert the regional ordering that the sources establish. One multiplier flexes the level and PRESERVES the ordering. Aggressive 1.35 puts the UAE at ~257, still under the AED 1,000 mark; conservative 0.70 puts it at ~133, below Botim's own sub-AED-500 majority. ASSUMPTION about spread, applied to observed levels.</t>
+          <t>REPLACED the global 'Average spot ticket' on 2026-08-21. The LEVEL is no longer a scenario input: each region now carries its own OBSERVED ticket on Assumptions (UAE 190 from Botim, India 40 from Augmont, Oman &amp; Bahrain 145 inferred). This parameter carries only the UNCERTAINTY around those observations, as a single dial. WHY ONE DIAL AND NOT THREE: three regional triplets would be nine numbers to defend and would let a scenario silently invert the regional ordering that the sources establish. One multiplier flexes the level and PRESERVES the ordering. Aggressive 1.35 puts the UAE at ~257, still under the AED 1,000 mark; conservative 0.70 puts it at ~133, below Botim's own sub-AED-500 majority. ASSUMPTION about spread, applied to observed levels.</t>
         </is>
       </c>
     </row>
@@ -5369,7 +5369,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>⚠ PROVENANCE CORRECTED 2026-08-21 - THE NUMBER STANDS, ITS OLD CITATION DID NOT. The previous note read 'Botim's 128,000 trades against ~45,000 buyers implies ~1.9/yr'. THE 45,000 IS NOT A BUYER COUNT, IT IS A TRANSACTION COUNT: Khaleej Times, Nov 2025, says 775,000 users EXPLORED the feature, 'completing over 45,000 transactions'. The 128,000 is also transactions, to Feb 2026. So the old derivation divided transactions by transactions across two different windows - the result was the growth in cumulative trades, not a frequency. CONFIRMED NEGATIVE: Botim has never published a unique-buyer count, so no frequency can be derived from it, and no published frequency exists ANYWHERE for ad-hoc lump gold purchases. Comparators are 0.85/yr (Augmont, per REGISTERED user, at an average transaction of Rs 331 - micro-saving, not lumps) and 264/yr (Jar, Rs 10/day auto-roundups) - a 300x spread, neither being this product. WHAT DOES SUPPORT 1.7 is a cross-check on the COMBINED basis, attach x frequency x ticket, which is comparable: Aurumix India implies ~Rs 838/yr of gold per paying customer against Augmont's ~Rs 281/yr per registered user. 3x, and defensible - our customers are engaged SIP savers, not dormant registrations. Behaviourally 1.7 is also about right for festive lumps: Dhanteras, Akshaya Tritiya and a wedding is roughly two events. ASSUMPTION, cross-checked on the combined basis, NOT directly sourced.</t>
+          <t>PROVENANCE CORRECTED 2026-08-21 - THE NUMBER STANDS, ITS OLD CITATION DID NOT. The previous note read 'Botim's 128,000 trades against ~45,000 buyers implies ~1.9/yr'. THE 45,000 IS NOT A BUYER COUNT, IT IS A TRANSACTION COUNT: Khaleej Times, Nov 2025, says 775,000 users EXPLORED the feature, 'completing over 45,000 transactions'. The 128,000 is also transactions, to Feb 2026. So the old derivation divided transactions by transactions across two different windows - the result was the growth in cumulative trades, not a frequency. CONFIRMED NEGATIVE: Botim has never published a unique-buyer count, so no frequency can be derived from it, and no published frequency exists ANYWHERE for ad-hoc lump gold purchases. Comparators are 0.85/yr (Augmont, per REGISTERED user, at an average transaction of Rs 331 - micro-saving, not lumps) and 264/yr (Jar, Rs 10/day auto-roundups) - a 300x spread, neither being this product. WHAT DOES SUPPORT 1.7 is a cross-check on the COMBINED basis, attach x frequency x ticket, which is comparable: Aurumix India implies ~Rs 838/yr of gold per paying customer against Augmont's ~Rs 281/yr per registered user. 3x, and defensible - our customers are engaged SIP savers, not dormant registrations. Behaviourally 1.7 is also about right for festive lumps: Dhanteras, Akshaya Tritiya and a wedding is roughly two events. ASSUMPTION, cross-checked on the combined basis, NOT directly sourced.</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5472,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-20, client decision: THE CARD IS A DRAWDOWN ON THE GOLD-COLLATERALISED FACILITY, not a salary-repaid revolving card. Aurumix has no balance sheet to lend from - it can only extend credit against collateral it holds, which is the customer's gold. Using the card IS borrowing, so card activation and credit take-up are the SAME behaviour and were previously modelled as two different populations (50% activating a card, 18% taking credit) doing what is in fact one thing. Merged onto the credit figure, which is the better-anchored of the two: Indian gold-loan penetration is under 10% at a point in time, uplifted here for pre-selection since these customers have already cleared a six-payment gate. ⚠ THE OLD 50% CAME FROM NEOBANK COMPARABLES (PULSE 68.2%, Monzo 68%) WHERE THE CARD IS THE PRODUCT - wrong in kind for a card that only lets you borrow against your own savings. DERIVED.</t>
+          <t>RE-BASED 2026-08-20, client decision: THE CARD IS A DRAWDOWN ON THE GOLD-COLLATERALISED FACILITY, not a salary-repaid revolving card. Aurumix has no balance sheet to lend from - it can only extend credit against collateral it holds, which is the customer's gold. Using the card IS borrowing, so card activation and credit take-up are the SAME behaviour and were previously modelled as two different populations (50% activating a card, 18% taking credit) doing what is in fact one thing. Merged onto the credit figure, which is the better-anchored of the two: Indian gold-loan penetration is under 10% at a point in time, uplifted here for pre-selection since these customers have already cleared a six-payment gate. THE OLD 50% CAME FROM NEOBANK COMPARABLES (PULSE 68.2%, Monzo 68%) WHERE THE CARD IS THE PRODUCT - wrong in kind for a card that only lets you borrow against your own savings. DERIVED.</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>RE-BASED 2026-08-20 from 12 transactions/MONTH once the card became a drawdown on the gold facility. Under that model the customer borrows a lump (limit x drawn share) a couple of times a year and spends it down, so the meaningful unit is transactions PER DRAW, not per month. At 12/month the implied ticket collapsed to ~AED 12, which is a coffee, not a reason to pledge your gold. THE AVERAGE TICKET FALLS OUT AS drawn amount / this number, and the draw events cancel - so the ticket depends only on how large a draw is and how many purchases it is spent across. ⚠ IT ALSO CHANGES WHAT THE CARD IS FOR: not daily groceries, but occasional larger needs - school fees, a medical bill, an emergency - funded by borrowing against savings rather than liquidating them. That is a materially different product story and should be put to the client in those words. ASSUMPTION.</t>
+          <t>RE-BASED 2026-08-20 from 12 transactions/MONTH once the card became a drawdown on the gold facility. Under that model the customer borrows a lump (limit x drawn share) a couple of times a year and spends it down, so the meaningful unit is transactions PER DRAW, not per month. At 12/month the implied ticket collapsed to ~AED 12, which is a coffee, not a reason to pledge your gold. THE AVERAGE TICKET FALLS OUT AS drawn amount / this number, and the draw events cancel - so the ticket depends only on how large a draw is and how many purchases it is spent across. IT ALSO CHANGES WHAT THE CARD IS FOR: not daily groceries, but occasional larger needs - school fees, a medical bill, an emergency - funded by borrowing against savings rather than liquidating them. That is a materially different product story and should be put to the client in those words. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>SET AT 0.15 on 2026-08-21, client instruction - the same day it came DOWN from 0.20 to 0.08, so it has landed close to where it started. What has genuinely changed is not the number but the STRUCTURE. ⚠ THE UNIT ALSO CHANGED, AND THAT MATTERS: it is now the share of NEW customers who take the plan when they join, feeding a SUBSCRIBER BALANCE that then churns - not a standing share of the whole book that could never fall. The steady-state share of paying customers holding a plan therefore lands BELOW this number. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on; 20% is at the top of the normal range for an OPTIONAL PAID extra on a savings product, which is low single digits to low teens. ⚠ IT IS NOT EQUIVALENT TO THE OLD 20% AND SHOULD NOT BE READ AS A PARTIAL REVERSAL: 20% was a permanent share of the whole book that could never decay, while 15% applies once, on joining, to a balance that then churns at ~7.1% a month. The standing share of paying customers holding a plan settles near 10.5%, not 15%. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on. ASSUMPTION.</t>
+          <t>SET AT 0.15 on 2026-08-21, client instruction - the same day it came DOWN from 0.20 to 0.08, so it has landed close to where it started. What has genuinely changed is not the number but the STRUCTURE. THE UNIT ALSO CHANGED, AND THAT MATTERS: it is now the share of NEW customers who take the plan when they join, feeding a SUBSCRIBER BALANCE that then churns - not a standing share of the whole book that could never fall. The steady-state share of paying customers holding a plan therefore lands BELOW this number. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on; 20% is at the top of the normal range for an OPTIONAL PAID extra on a savings product, which is low single digits to low teens. IT IS NOT EQUIVALENT TO THE OLD 20% AND SHOULD NOT BE READ AS A PARTIAL REVERSAL: 20% was a permanent share of the whole book that could never decay, while 15% applies once, on joining, to a balance that then churns at ~7.1% a month. The standing share of paying customers holding a plan settles near 10.5%, not 15%. NOTHING IS STATED ANYWHERE IN THE CORPUS and no attach benchmark exists for this kind of add-on. ASSUMPTION.</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>ADDED 2026-08-21. THE FIRST IS INCLUDED IN THE PLAN PRICE, so only the excess over 1.0 is charged - at 2.5 that is 1.5 chargeable. No platform publishes beneficiaries-per-will. What anchors it is who these customers are: South Asian migrant workers who remit ~80% of income to families at home, typically supporting a spouse, children and parents. Household sizes in the source countries run ~4.4 in India, ~4.5 in Bangladesh and ~6.8 in Pakistan, so naming 2-3 beneficiaries is conservative against the family they actually support. ⚠ NOT THE SAME AS HOUSEHOLD SIZE - a beneficiary is a named, identity-verified person on a legal instrument, and people name fewer than they support. ASSUMPTION anchored on demographics.</t>
+          <t>ADDED 2026-08-21. THE FIRST IS INCLUDED IN THE PLAN PRICE, so only the excess over 1.0 is charged - at 2.5 that is 1.5 chargeable. No platform publishes beneficiaries-per-will. What anchors it is who these customers are: South Asian migrant workers who remit ~80% of income to families at home, typically supporting a spouse, children and parents. Household sizes in the source countries run ~4.4 in India, ~4.5 in Bangladesh and ~6.8 in Pakistan, so naming 2-3 beneficiaries is conservative against the family they actually support. NOT THE SAME AS HOUSEHOLD SIZE - a beneficiary is a named, identity-verified person on a legal instrument, and people name fewer than they support. ASSUMPTION anchored on demographics.</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6106,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6196,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6286,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. ⚠ THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
+          <t>RAISED 2026-08-21. Base now reaches 11 by Y7, against ~20 nameable Gulf candidates without a gold product - roughly a 55% win rate on the addressable partner market, which is aggressive but arguable for a category with one incumbent. Partner 1 signs in Y2, matching the M13 B2B go-live. THE CANDIDATE LIST IS THE JUSTIFICATION AND IT IS FINITE: e&amp; money, Payit, Careem Pay, Al Ansari, LuLu Money, Rise, NOW Money, Wio, Liv, Mashreq Neo, Klip, PayBy, Jingle Pay, Thawani, BenefitPay, CWallet, Amanat and a handful of banks and exchange houses. Going much above this count means claiming partners that have not been named. ASSUMPTION on a sourced candidate set.</t>
         </is>
       </c>
     </row>
@@ -6316,7 +6316,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>THE MIX, NOT THE BIGGEST. A realistic six-partner Gulf book is roughly one Botim-scale (1.7m ACTIVE fintech users, of 8.2-8.5m app users), two at e&amp; money scale (~1.5m subscribers), and three small wallets at a few hundred thousand - which averages near 900k. ⚠ USE ACTIVE USERS, NOT REGISTERED: Botim's own numbers separate 8.5m app users, 3m KYC'd and 1.7m active fintech users, and adopting the headline would overstate this by 5x. CITED for the two largest, ASSUMPTION for the tail.</t>
+          <t>THE MIX, NOT THE BIGGEST. A realistic six-partner Gulf book is roughly one Botim-scale (1.7m ACTIVE fintech users, of 8.2-8.5m app users), two at e&amp; money scale (~1.5m subscribers), and three small wallets at a few hundred thousand - which averages near 900k. USE ACTIVE USERS, NOT REGISTERED: Botim's own numbers separate 8.5m app users, 3m KYC'd and 1.7m active fintech users, and adopting the headline would overstate this by 5x. CITED for the two largest, ASSUMPTION for the tail.</t>
         </is>
       </c>
     </row>
@@ -6346,7 +6346,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>OBSERVED ANCHOR: O Gold reports 75,000 ACTIVE users against Botim's 1.7m active fintech users - 4.4% - and 775,000 who merely explored the feature. Base is set at 6%, ABOVE the observed 4.4%, because that figure is roughly six months after the gold feature launched and adoption should mature; 6% is a 1.4x maturation, not a doubling. ⚠ THE 4.4% IS THE ONLY OBSERVED GOLD-ADOPTION RATE FOR A GULF WALLET THAT EXISTS. TRIANGULATED.</t>
+          <t>OBSERVED ANCHOR: O Gold reports 75,000 ACTIVE users against Botim's 1.7m active fintech users - 4.4% - and 775,000 who merely explored the feature. Base is set at 6%, ABOVE the observed 4.4%, because that figure is roughly six months after the gold feature launched and adoption should mature; 6% is a 1.4x maturation, not a doubling. THE 4.4% IS THE ONLY OBSERVED GOLD-ADOPTION RATE FOR A GULF WALLET THAT EXISTS. TRIANGULATED.</t>
         </is>
       </c>
     </row>
@@ -8409,7 +8409,7 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>⚠ RISING GOLD CUTS BOTH WAYS AND THE MODEL CAPTURES BOTH. Metal already held appreciates, but a fixed USD contribution BUYS FEWER GRAMS each year - so AUM does NOT simply compound at the headline rate. Only the collateral-linked streams move with this row (card limit, and lending through it); the entry fee is a percentage of a USD contribution and is untouched by the gold price.</t>
+          <t>RISING GOLD CUTS BOTH WAYS AND THE MODEL CAPTURES BOTH. Metal already held appreciates, but a fixed USD contribution BUYS FEWER GRAMS each year - so AUM does NOT simply compound at the headline rate. Only the collateral-linked streams move with this row (card limit, and lending through it); the entry fee is a percentage of a USD contribution and is untouched by the gold price.</t>
         </is>
       </c>
     </row>
@@ -24986,7 +24986,7 @@
     <row r="162">
       <c r="A162" s="9" t="inlineStr">
         <is>
-          <t>THE NUMBER TO QUOTE AGAINST OTHER GOLD PLATFORMS, and the only one that compares like for like. Collateral-eligible AUM above is SMALLER because it also removes gold moved out of Aurumix's control - a token in a private wallet cannot back a credit limit, but THE METAL IS STILL IN THE VAULT, so it is still gold under custody. PAXG, Kinesis and Comtech all publish the custody measure. ⚠ COMPARE IN GRAMS, NOT DOLLARS: every published USD figure carries the gold price of its own vintage, so a comparison in dollars is really a comparison of gold prices. Comtech Gold, the closest comparable - Dubai, DMCC-licensed, tokenised gold - holds ~141,000 g.</t>
+          <t>THE NUMBER TO QUOTE AGAINST OTHER GOLD PLATFORMS, and the only one that compares like for like. Collateral-eligible AUM above is SMALLER because it also removes gold moved out of Aurumix's control - a token in a private wallet cannot back a credit limit, but THE METAL IS STILL IN THE VAULT, so it is still gold under custody. PAXG, Kinesis and Comtech all publish the custody measure. COMPARE IN GRAMS, NOT DOLLARS: every published USD figure carries the gold price of its own vintage, so a comparison in dollars is really a comparison of gold prices. Comtech Gold, the closest comparable - Dubai, DMCC-licensed, tokenised gold - holds ~141,000 g.</t>
         </is>
       </c>
     </row>
@@ -25249,7 +25249,7 @@
     <row r="165">
       <c r="A165" s="9" t="inlineStr">
         <is>
-          <t>THE HONEST SERIES FOR JUDGING EXECUTION is the constant-price row: it strips the gold price out and leaves grams accumulated, which is the part Aurumix controls. The headline above will grow even if the business does not. ⚠ SET GOLD APPRECIATION TO THE CONSERVATIVE SCENARIO (0.0%) TO RECOVER THE ORIGINAL FLAT-PRICE MODEL, under which these two rows are identical by construction.</t>
+          <t>THE HONEST SERIES FOR JUDGING EXECUTION is the constant-price row: it strips the gold price out and leaves grams accumulated, which is the part Aurumix controls. The headline above will grow even if the business does not. SET GOLD APPRECIATION TO THE CONSERVATIVE SCENARIO (0.0%) TO RECOVER THE ORIGINAL FLAT-PRICE MODEL, under which these two rows are identical by construction.</t>
         </is>
       </c>
     </row>

</xml_diff>